<commit_message>
PCB rev 0.6: LCSC order list that matches 95/95 in the BOM tool
U20 becomes the RP2354B (C39843328): LCSC does not sell the RP2350B
outside China. U21 flash is marked not fitted and dropped from the JLC
BOM/CPL. Out-of-stock parts swapped for equivalents, lcsc_paste.txt added
for the BOM tool's Copy & Paste box, order instructions updated.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PCB/rev0.6/order/lcsc_cart_one_set_upload.xlsx
+++ b/PCB/rev0.6/order/lcsc_cart_one_set_upload.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -638,7 +638,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>C28260</t>
+          <t>C77060</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1013,12 +1013,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>C96895</t>
+          <t>C167882</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>18uH SWPA4030S180MT 18uH</t>
+          <t>18uH cjiang FNR4030S180MT 18uH 4x4mm shielded, Isat 1.5A, Irms 1.2A, 260 mOhm (SWPA4030S180MT C96895 discontinued at LCS</t>
         </is>
       </c>
     </row>
@@ -1114,16 +1114,16 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>C5116480</t>
+          <t>C19630936</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Main board plug ZHOURI 2.54-2*10 male pin header</t>
+          <t>Main board plug 2x8 2.54mm male pin header</t>
         </is>
       </c>
     </row>
@@ -1133,12 +1133,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>C30867</t>
+          <t>C5116480</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>USB module socket BOOMELE 2.54-2*10P female 8.5mm (LCSC out of stock 2026-10-01; any 2x10 2.54mm 8.5mm socket fits)</t>
+          <t>Main board plug ZHOURI 2.54-2*10 male pin header</t>
         </is>
       </c>
     </row>
@@ -1148,192 +1148,192 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>C42415655</t>
+          <t>C239344</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>RP2350B Raspberry Pi RP2350B QFN-80 (LCSC stock unclear; alt RP2354B C39843328 with 2MB internal flash, then leave U21 u</t>
+          <t>K-line module socket CJT A2541HWV-2x4P 2x4 2.54mm female socket, 8.5mm body</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>C4154405</t>
+          <t>C22440830</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>CH334R WCH CH334R 4-port USB 2.0 hub, QSOP-16</t>
+          <t>GNSS module socket kinghelm KH-2.54FH-2X8P-H8.5 2x8 2.54mm female socket, 8.5mm body</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>C17168</t>
+          <t>C5821035</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0ohm UNI-ROYAL 0402WGF0000TCE 0402 0R</t>
+          <t>USB module socket CJT A2541HWV-2x10P 2x10 2.54mm female socket, 8.5mm body</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>C25803</t>
+          <t>C39843328</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>100k 0603 100k 1%</t>
+          <t>RP2354B Raspberry Pi RP2354B QFN-80 (RP2350B with 2 MB flash in the package; the RP2350B C42415655 is not sold outside C</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>C23352</t>
+          <t>C4154405</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>24k 0603 24k 1%</t>
+          <t>CH334R WCH CH334R 4-port USB 2.0 hub, QSOP-16</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>C23162</t>
+          <t>C17168</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>4.7k 0603 4.7k 1%</t>
+          <t>0ohm UNI-ROYAL 0402WGF0000TCE 0402 0R</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>C25804</t>
+          <t>C25803</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>10k 0603 10k 1%</t>
+          <t>100k 0603 100k 1%</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>C22775</t>
+          <t>C23352</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>100ohm 0603 100 1%</t>
+          <t>24k 0603 24k 1%</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>C21190</t>
+          <t>C23162</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>1k 0603 1k 1%</t>
+          <t>4.7k 0603 4.7k 1%</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>C22935</t>
+          <t>C98220</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>1M 0603 1M 1%</t>
+          <t>10k YAGEO RC0603FR-0710KL 0603 10k 1%</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>C22961</t>
+          <t>C22775</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>220k 0603 220k 1%</t>
+          <t>100ohm 0603 100 1%</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>C23140</t>
+          <t>C21190</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>33ohm 0603 33 1%</t>
+          <t>1k 0603 1k 1%</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>C21189</t>
+          <t>C22935</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>0ohm 0603 0 1%</t>
+          <t>1M 0603 1M 1%</t>
         </is>
       </c>
     </row>
@@ -1343,57 +1343,57 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>C105579</t>
+          <t>C22961</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>47k 0603 47k 1% (YAGEO RC0603FR-0747KL)</t>
+          <t>220k 0603 220k 1%</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>C22984</t>
+          <t>C23140</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>30k UNI-ROYAL 0603WAF3002T5E</t>
+          <t>33ohm 0603 33 1%</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>C25981</t>
+          <t>C21189</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>8.2k 0603 8.2k 1%</t>
+          <t>0ohm 0603 0 1%</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>C25190</t>
+          <t>C105579</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>27ohm 0603 27 1%</t>
+          <t>47k 0603 47k 1% (YAGEO RC0603FR-0747KL)</t>
         </is>
       </c>
     </row>
@@ -1403,12 +1403,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>C13564</t>
+          <t>C22984</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>NTC 10k B3950 Murata NCP18XH103F03RB 10k B3380 0603</t>
+          <t>30k UNI-ROYAL 0603WAF3002T5E</t>
         </is>
       </c>
     </row>
@@ -1418,12 +1418,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>C22859</t>
+          <t>C25981</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>10ohm 0603 10 1%</t>
+          <t>8.2k 0603 8.2k 1%</t>
         </is>
       </c>
     </row>
@@ -1433,12 +1433,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>C23179</t>
+          <t>C25190</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>470ohm 0603 470 1%</t>
+          <t>27ohm 0603 27 1%</t>
         </is>
       </c>
     </row>
@@ -1448,87 +1448,87 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>C23153</t>
+          <t>C13564</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>39k 0603 39k 1%</t>
+          <t>NTC 10k B3950 Murata NCP18XH103F03RB 10k B3380 0603</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>C17673</t>
+          <t>C22859</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>4.7kohm 0805 0805 4.7k 1%</t>
+          <t>10ohm 0603 10 1%</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>C17521</t>
+          <t>C23179</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2.2ohm 0805 UNI-ROYAL 0805W8F220KT5E 0805 2.2R 125mW</t>
+          <t>470ohm 0603 470 1%</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>C375691</t>
+          <t>C23153</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>10mohm 2512 Yageo PA2512FKE7T0R01E 10 mOhm 1% 3W</t>
+          <t>39k 0603 39k 1%</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>C470884</t>
+          <t>C17673</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>EL817S1(C) EL817S1(C)(TU)-F (EL817S1(C)(TU)-FV)</t>
+          <t>4.7kohm 0805 0805 4.7k 1%</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>C97521</t>
+          <t>C17521</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>W25Q128JVS Winbond W25Q128JVSIQ</t>
+          <t>2.2ohm 0805 UNI-ROYAL 0805W8F220KT5E 0805 2.2R 125mW</t>
         </is>
       </c>
     </row>
@@ -1538,27 +1538,27 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>C400792</t>
+          <t>C375691</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>P-MOSFET -60V onsemi FDN5618P -60V P-MOSFET (check 1=G 2=S 3=D in datasheet)</t>
+          <t>10mohm 2512 Yageo PA2512FKE7T0R01E 10 mOhm 1% 3W</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>C8545</t>
+          <t>C109227</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2N7002 JSCJ 2N7002</t>
+          <t>EL817S1(C) EL817S1(C)(TU)-F (EL817S1(C)(TU)-FV)</t>
         </is>
       </c>
     </row>
@@ -1568,27 +1568,27 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>C20917</t>
+          <t>C400792</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>AO3400A AO3400A 30V 5.7A N-MOSFET</t>
+          <t>P-MOSFET -60V onsemi FDN5618P -60V P-MOSFET (check 1=G 2=S 3=D in datasheet)</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>C5370990</t>
+          <t>C8545</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>LP5907MFX-3.3 TI LP5907MFX-3.3/NOPB 250mA LDO (TECH PUBLIC TPLP5907MFX-3.3 clone; TI part out of stock at LCSC)</t>
+          <t>2N7002 JSCJ 2N7002</t>
         </is>
       </c>
     </row>
@@ -1598,87 +1598,87 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>C51118</t>
+          <t>C20917</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>AP2112K-3.3 Diodes AP2112K-3.3TRG1</t>
+          <t>AO3400A AO3400A 30V 5.7A N-MOSFET</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>C524782</t>
+          <t>C5370990</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>TPS560430XDBVR TPS560430XDBVR 36V 600mA buck, 1.1MHz</t>
+          <t>LP5907MFX-3.3 TI LP5907MFX-3.3/NOPB 250mA LDO (TECH PUBLIC TPLP5907MFX-3.3 clone; TI part out of stock at LCSC)</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>C7519</t>
+          <t>C51118</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>USBLC6-2SC6 ST USBLC6-2SC6</t>
+          <t>AP2112K-3.3 Diodes AP2112K-3.3TRG1</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>C2886898</t>
+          <t>C524782</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>RESET E-Switch TL3342F160QG</t>
+          <t>TPS560430XDBVR TPS560430XDBVR 36V 600mA buck, 1.1MHz</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>C841384</t>
+          <t>C7519</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>LMR33630ADDA TI LMR33630ADDAR 36V 3A buck, 400 kHz</t>
+          <t>USBLC6-2SC6 ST USBLC6-2SC6</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>C130101</t>
+          <t>C2886898</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>P-MOSFET -40V NCE40P70K -40V 10 mOhm P-MOSFET TO-252 (alt Diodes DMP4015SK3-13 C513222)</t>
+          <t>RESET E-Switch TL3342F160QG</t>
         </is>
       </c>
     </row>
@@ -1688,27 +1688,27 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>C2864583</t>
+          <t>C841384</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>TPS55288RPMR TI TPS55288RPMR</t>
+          <t>LMR33630ADDA TI LMR33630ADDAR 36V 3A buck, 400 kHz</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>C107671</t>
+          <t>C130101</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>PCM5102APWR TI PCM5102APWR 32-bit 384kHz stereo DAC</t>
+          <t>P-MOSFET -40V NCE40P70K -40V 10 mOhm P-MOSFET TO-252 (alt Diodes DMP4015SK3-13 C513222)</t>
         </is>
       </c>
     </row>
@@ -1718,27 +1718,27 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>C88374</t>
+          <t>C2864583</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>U.FL GNSS antenna Hirose U.FL-R-SMT-1(80) U.FL receptacle; antenna via U.FL-to-SMA pigtail</t>
+          <t>TPS55288RPMR TI TPS55288RPMR</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>C2798029</t>
+          <t>C107671</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>External USB 2 Molex 67643-0910 USB-A</t>
+          <t>PCM5102APWR TI PCM5102APWR 32-bit 384kHz stereo DAC</t>
         </is>
       </c>
     </row>
@@ -1748,27 +1748,27 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>C140303</t>
+          <t>C88374</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>TPS2561DRCR TI TPS2561DRCR dual 2.8A USB power switch</t>
+          <t>U.FL GNSS antenna Hirose U.FL-R-SMT-1(80) U.FL receptacle; antenna via U.FL-to-SMA pigtail</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>C840100</t>
+          <t>C2798029</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>CSD18543Q3A TI CSD18543Q3A 60V 8.5mOhm N-MOSFET</t>
+          <t>External USB 2 Molex 67643-0910 USB-A</t>
         </is>
       </c>
     </row>
@@ -1778,27 +1778,27 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>C2856837</t>
+          <t>C140303</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Display FPC 40P 0.5mm XUNPU FPC-05FB-40PH20, 40P 0.5mm dual-contact flip-top 2.0mm (pads numbered by panel pin: pin 1 on</t>
+          <t>TPS2561DRCR TI TPS2561DRCR dual 2.8A USB power switch</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>C5119087</t>
+          <t>C840100</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>NEO-M9N-00B u-blox NEO-M9N-00B</t>
+          <t>CSD18543Q3A TI CSD18543Q3A 60V 8.5mOhm N-MOSFET</t>
         </is>
       </c>
     </row>
@@ -1808,12 +1808,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>C178942</t>
+          <t>C2856837</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Littelfuse 029707.5WXNV 7.5A mini blade fuse for holder F4</t>
+          <t>Display FPC 40P 0.5mm XUNPU FPC-05FB-40PH20, 40P 0.5mm dual-contact flip-top 2.0mm (pads numbered by panel pin: pin 1 on</t>
         </is>
       </c>
     </row>
@@ -1823,10 +1823,40 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
+          <t>C5119087</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>NEO-M9N-00B u-blox NEO-M9N-00B</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>1</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>C178942</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Littelfuse 029707.5WXNV 7.5A mini blade fuse for holder F4</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>1</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
           <t>C5305</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr">
+      <c r="C96" t="inlineStr">
         <is>
           <t>2.54 mm jumper cap for JP1</t>
         </is>

</xml_diff>

<commit_message>
PCB rev 0.6: USB module L4 Bourns SRP6060FA-8R2M instead of Coilcraft XAL6060
Same 8.2 uH / 8.5 A Isat / 22.5 mOhm and the same land pattern, $1.38
instead of $12.34. LCSC cart, paste list and order notes updated.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PCB/rev0.6/order/lcsc_cart_one_set_upload.xlsx
+++ b/PCB/rev0.6/order/lcsc_cart_one_set_upload.xlsx
@@ -983,12 +983,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>C19191627</t>
+          <t>C2045598</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>8.2uH 5A Coilcraft XAL6060-822MEC 8.2uH Isat 8.4A 24 mOhm (expensive; any 8.2-10uH shielded, Isat &gt;= 5A works)</t>
+          <t>8.2uH 5A Bourns SRP6060FA-8R2M 8.2uH Isat 8.5A Irms 6A 22.5 mOhm (same land pattern as the Coilcraft XAL6060-822MEC foot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
PCB rev 0.6: VIM3 power key through a PhotoMOS (U22, AQY210S)
U22 shorts the two J5 pins (the VIM3 POWER key pads), isolated, instead of
Q1 pulling J5 pin 1 to GND. It sits on the bottom side next to J5; R12 is
now the 390 ohm LED resistor from GPIO15, R19 is gone. Schematic, board,
order files, LCSC list and docs updated. DRC: 0 unconnected, no errors.
bridge.py vias now use the board's 0.3 mm drill. A stale KiCad lock file is
untracked and *.lck ignored.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PCB/rev0.6/order/lcsc_cart_one_set_upload.xlsx
+++ b/PCB/rev0.6/order/lcsc_cart_one_set_upload.xlsx
@@ -1234,7 +1234,7 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -1294,7 +1294,7 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -1354,46 +1354,46 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>C23140</t>
+          <t>C23151</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>33ohm 0603 33 1%</t>
+          <t>390ohm UNI-ROYAL 0603WAF3900T5E 390 1%</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>C21189</t>
+          <t>C23140</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>0ohm 0603 0 1%</t>
+          <t>33ohm 0603 33 1%</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>C105579</t>
+          <t>C21189</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>47k 0603 47k 1% (YAGEO RC0603FR-0747KL)</t>
+          <t>0ohm 0603 0 1%</t>
         </is>
       </c>
     </row>
@@ -1403,12 +1403,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>C22984</t>
+          <t>C105579</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>30k UNI-ROYAL 0603WAF3002T5E</t>
+          <t>47k 0603 47k 1% (YAGEO RC0603FR-0747KL)</t>
         </is>
       </c>
     </row>
@@ -1418,42 +1418,42 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>C25981</t>
+          <t>C22984</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>8.2k 0603 8.2k 1%</t>
+          <t>30k UNI-ROYAL 0603WAF3002T5E</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>C25190</t>
+          <t>C25981</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>27ohm 0603 27 1%</t>
+          <t>8.2k 0603 8.2k 1%</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>C13564</t>
+          <t>C25190</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>NTC 10k B3950 Murata NCP18XH103F03RB 10k B3380 0603</t>
+          <t>27ohm 0603 27 1%</t>
         </is>
       </c>
     </row>
@@ -1463,117 +1463,117 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>C22859</t>
+          <t>C13564</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>10ohm 0603 10 1%</t>
+          <t>NTC 10k B3950 Murata NCP18XH103F03RB 10k B3380 0603</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>C23179</t>
+          <t>C22859</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>470ohm 0603 470 1%</t>
+          <t>10ohm 0603 10 1%</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>C23153</t>
+          <t>C23179</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>39k 0603 39k 1%</t>
+          <t>470ohm 0603 470 1%</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>C17673</t>
+          <t>C23153</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>4.7kohm 0805 0805 4.7k 1%</t>
+          <t>39k 0603 39k 1%</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>C17521</t>
+          <t>C17673</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2.2ohm 0805 UNI-ROYAL 0805W8F220KT5E 0805 2.2R 125mW</t>
+          <t>4.7kohm 0805 0805 4.7k 1%</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>C375691</t>
+          <t>C17521</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>10mohm 2512 Yageo PA2512FKE7T0R01E 10 mOhm 1% 3W</t>
+          <t>2.2ohm 0805 UNI-ROYAL 0805W8F220KT5E 0805 2.2R 125mW</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>C109227</t>
+          <t>C375691</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>EL817S1(C) EL817S1(C)(TU)-F (EL817S1(C)(TU)-FV)</t>
+          <t>10mohm 2512 Yageo PA2512FKE7T0R01E 10 mOhm 1% 3W</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>C400792</t>
+          <t>C109227</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>P-MOSFET -60V onsemi FDN5618P -60V P-MOSFET (check 1=G 2=S 3=D in datasheet)</t>
+          <t>EL817S1(C) EL817S1(C)(TU)-F (EL817S1(C)(TU)-FV)</t>
         </is>
       </c>
     </row>
@@ -1583,12 +1583,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>C8545</t>
+          <t>C400792</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2N7002 JSCJ 2N7002</t>
+          <t>P-MOSFET -60V onsemi FDN5618P -60V P-MOSFET (check 1=G 2=S 3=D in datasheet)</t>
         </is>
       </c>
     </row>
@@ -1598,12 +1598,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>C20917</t>
+          <t>C8545</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>AO3400A AO3400A 30V 5.7A N-MOSFET</t>
+          <t>2N7002 JSCJ 2N7002</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
PCB rev 0.6: LCSC list includes the cable-side connectors
Micro-Fit housings and crimps for the J1/J8 ISO pigtails and JST-PH
housings and crimps for J5/J7/J12; the order notes list the cables to buy
elsewhere.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PCB/rev0.6/order/lcsc_cart_one_set_upload.xlsx
+++ b/PCB/rev0.6/order/lcsc_cart_one_set_upload.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C96"/>
+  <dimension ref="A1:C103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -1862,6 +1862,111 @@
         </is>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>5</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>C127351</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Molex 43025-0800 Micro-Fit 2x4 plug housing for J1 (ISO A pigtail), min 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>5</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>C293525</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Molex 43025-0600 Micro-Fit 2x3 plug housing for J8 (ISO C1 pigtail), min 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>20</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>C293530</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Molex 43030-0007 Micro-Fit crimp 20-24 AWG for J1/J8 (14 used)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>50</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>C157955</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>JST PHR-2 housing for J5 (VIM3 power key), min 50</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>50</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>C111514</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>JST PHR-4 housing for J7 (light sensor), min 50</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>20</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>C157953</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>JST PHR-5 housing for J12 (display buttons), min 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>100</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>C111515</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>JST SPH-002T-P0.5S PH crimp 24-30 AWG for J5/J7/J12 (11 used), min 100</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>